<commit_message>
Update mock excel script for easier user input
</commit_message>
<xml_diff>
--- a/participants.xlsx
+++ b/participants.xlsx
@@ -453,12 +453,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jash</t>
+          <t>Name A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>jash@example.com</t>
+          <t>your_first_email@company.com</t>
         </is>
       </c>
     </row>
@@ -470,12 +470,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chinnmay</t>
+          <t>Name B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>chinnmay@example.com</t>
+          <t>your_second_email@company.com</t>
         </is>
       </c>
     </row>
@@ -487,12 +487,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Name C</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>alice.test@example.com</t>
+          <t>your_third_email@company.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Expand master participant list with 8 speakers
</commit_message>
<xml_diff>
--- a/participants.xlsx
+++ b/participants.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,12 +453,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Name A</t>
+          <t>alex</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>your_first_email@company.com</t>
+          <t>learningtraverse@gmail.com</t>
         </is>
       </c>
     </row>
@@ -470,12 +470,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Name B</t>
+          <t>jamie</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>your_second_email@company.com</t>
+          <t>lohithnandyal1@gmail.com</t>
         </is>
       </c>
     </row>
@@ -487,12 +487,97 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Name C</t>
+          <t>sam</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>your_third_email@company.com</t>
+          <t>leematans05@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Speaker D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cassey</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>srujana.hm15@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Speaker E</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lohith</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dishahali075@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Speaker F</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>shreya</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nandyallohith@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Speaker G</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>samruddhi</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>samruddhims1111@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Speaker H</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gagan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>shreyaanadkumar3@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>